<commit_message>
Reprova três lojas de TCG na triagem e faz a análise de conteúdo (Bardin) do Bloco B
Bolsa do Infinito, Polar Jogos e PlayGround Game Store saem dos aprovados:
nova conferência das fotos deixou dúvida e o Instagram confirmou lojas de TCG.

A análise de conteúdo codifica os 575 comentários válidos da base do Notion
(livro de códigos, regras de decisão, tipologia casa de jogos x loja) e o
script gera as frequências e a amostra estratificada de 112 comentários para
a recodificação cega de controle.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_data/processed/[A] Estabelecimentos e cardapios/bloco_b_triagem_manual_metropoles_mais_100_avaliacoes.xlsx
+++ b/_data/processed/[A] Estabelecimentos e cardapios/bloco_b_triagem_manual_metropoles_mais_100_avaliacoes.xlsx
@@ -7385,37 +7385,37 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>insuficientes</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>não</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>não se aplica</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>não se aplica</t>
+          <t>não</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>luderia</t>
+          <t>loja de TCG</t>
         </is>
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>aprovado</t>
+          <t>reprovado</t>
         </is>
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t>luderia autentica</t>
+          <t>instagram, loja de TCG</t>
         </is>
       </c>
     </row>
@@ -9400,37 +9400,37 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>insuficientes</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>não</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>não se aplica</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>não se aplica</t>
+          <t>não</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
         <is>
-          <t>luderia</t>
+          <t>loja de TCG</t>
         </is>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>aprovado</t>
+          <t>reprovado</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>luderia autentica</t>
+          <t>instagram, loja de TCG</t>
         </is>
       </c>
     </row>
@@ -10365,37 +10365,37 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>insuficientes</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>não</t>
         </is>
       </c>
       <c r="L134" t="inlineStr">
         <is>
-          <t>não se aplica</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>não se aplica</t>
+          <t>não</t>
         </is>
       </c>
       <c r="N134" t="inlineStr">
         <is>
-          <t>luderia</t>
+          <t>loja de TCG</t>
         </is>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>aprovado</t>
+          <t>reprovado</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>luderia autentica</t>
+          <t>instagram, loja de TCG</t>
         </is>
       </c>
     </row>

</xml_diff>